<commit_message>
feat(F-NAR-019): ATOM-COL.POL.001-06 La pomme et la tulipe de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.POL.001-06.xlsx
+++ b/stories/arbres/ATOM-COL.POL.001-06.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La pomme et la tulipe de Victorino</t>
+          <t>La pomme et la tulipe de Nino</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>épicerie du chat gris, puis fleuriste</t>
+          <t>épicerie puis fleuriste. Volet vert, caisse de pommes, pas de la porte, cloche de cuivre, tulipes dans l'eau</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorino, papa, maman</t>
+          <t>Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorino veut la pomme à joue rose, puis une tulipe pour la table. Il dit bonjour, s'il te plaît, merci aux deux dames. La tulipe tient dans le verre.</t>
+          <t>Une poussière claire tombe du volet vert. Sur le bois, un éclat de volet luit. Nino veut la pomme à joue rose, maintenant. Il parle trop vite : les mots se cognent au bois. La dame ne lève pas les yeux. Sourire parti. Papa se baisse. Bonjour, s'il te plaît, merci vécus. Chez les fleurs, la tige glisse. Il refuse de foncer. Sur le bois, l'éclat de volet tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un chat gris se tient sur le pas. Il cligne, tout lent. Une caisse de pommes sent le sucré. Les pommes sont jaunes, avec un point rose. Un volet tape tout doux dans le vent. Le chat te regarde, Victorino. Il a des yeux jaunes. Comme les pommes. Une cloche de cuivre attend au-dessus de la porte. En ce moment, Victorino pousse un peu. La cloche fait ding. L'air dedans est frais, un peu sucré. Des bocaux brillent sur une étagère. Une pomme, maman. Celle à joue rose. On s'approche du comptoir. La dame essuie le bois du comptoir. Le chiffon sent le citron. Elle a le chiffon à la main. Victorino s'arrête devant les pommes. Le point rose brille sous la lampe. Un rayon touche le verre des bocaux. La dame pose le chiffon. Elle lève les yeux. Tu demandes, Victorino.</t>
+          <t>Une poussière claire tombe du volet vert. Le bois sent le soleil, un peu chaud. Sur le bois, un éclat de volet luit. Il brille, papa. Tu le vois, sur le volet ? Un chat gris se tient sur le pas. Il cligne, les yeux jaunes. Il me regarde, maman. Comme les pommes. Une caisse de pommes attend près du pas de la porte. Les pommes sont jaunes, avec une joue rose. Ça sent le sucré et le bois sec. Elles brillent, maman. Tu les vois, Nino ? Oui, maman. On avance. La cloche de cuivre penche au-dessus du bois. Papa pousse un peu le bois. En ce moment, Nino pousse un peu la porte. La cloche de cuivre fait ding. L'air dedans est frais, un peu sucré. Des bocaux brillent sur une étagère. Je la veux, maintenant. Celle à joue rose ? Oui, tout de suite ! La dame essuie le bois du comptoir. Le chiffon glisse, sans un bruit. Nino se dresse sur les pointes. Une pomme ! Les mots de Nino se cognent au bois. La dame ne lève pas les yeux. Ses mains sont pleines de chiffon. Oh. L'éclat de volet tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Elle ne me voit pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. La pomme est derrière le bois ? Oui, papa. Nino montre la pomme jaune, à joue rose. Tu parles à la dame, Nino. Le chiffon se pose enfin. La dame lève les yeux. Elle est là. Elle te regarde, Nino ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un chat gris se tient sur le pas. Il cligne, tout lent. Une caisse de pommes sent le sucré. Les pommes sont jaunes, avec un point rose. Un volet tape tout doux dans le vent. Le chat te regarde, Victorino. Il a des yeux jaunes. Comme les pommes. Une cloche de cuivre attend au-dessus de la porte. En ce moment, Victorino pousse un peu. La cloche fait ding. L'air dedans est frais, un peu sucré. Des bocaux brillent sur une étagère. Une pomme, maman. Celle à joue rose. On s'approche du comptoir. La dame essuie le bois du comptoir. Le chiffon sent le citron. Elle a le chiffon à la main. Victorino s'arrête devant les pommes. Le point rose brille sous la lampe. Un rayon touche le verre des bocaux. La dame pose le chiffon. Elle lève les yeux. Tu demandes, Victorino.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une poussière claire tombe du volet vert. Le bois sent le soleil, un peu chaud. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de volet&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le volet ? Un chat gris se tient sur le pas. Il cligne, les yeux jaunes. Il me regarde, maman. Comme les pommes. Une caisse de pommes attend près du pas de la porte. Les pommes sont jaunes, avec une joue rose. Ça sent le sucré et le bois sec. Elles brillent, maman. Tu les vois, Nino ? Oui, maman. On avance. La cloche de cuivre penche au-dessus du bois. Papa pousse un peu le bois. En ce moment, Nino pousse un peu la porte. La cloche de cuivre fait ding. L'air dedans est frais, un peu sucré. Des bocaux brillent sur une étagère. Je la veux, maintenant. Celle à joue rose ? Oui, tout de suite ! La dame essuie le bois du comptoir. Le chiffon glisse, sans un bruit. Nino se dresse sur les pointes. Une pomme ! Les mots de Nino se cognent au bois. La dame ne lève pas les yeux. Ses mains sont pleines de chiffon. Oh. L'éclat de volet tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Elle ne me voit pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. La pomme est derrière le bois ? Oui, papa. Nino montre la pomme jaune, à joue rose. Tu parles à la dame, Nino. Le chiffon se pose enfin. La dame lève les yeux. Elle est là. Elle te regarde, Nino ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand entre à l'épicerie avec maman. Les pommes sentent le sucré. Il voit la dame des fruits. Ferdinand dit : &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. La dame sourit. Ferdinand veut une pomme. Il dit : s'il te plaît. La dame tend la pomme. Ferdinand dit : merci. Il touche la peau lisse. Plus tard, ils vont chez la fleuriste. Les fleurs sentent fort. Ferdinand voit la dame des fleurs. Il se souvient. Il dit : bonjour. Il dit : une fleur, s'il te plaît. La dame tend une tulipe. Ferdinand dit : merci. Maman sourit. Même leçon, autre lieu. On salue. On demande. On remercie. Ferdinand porte la pomme et la tulipe. [pause]</t>
+          <t>Une poussière claire tombe du volet vert. Le bois sent le soleil, un peu chaud. Sur le bois, un &lt;emphasis&gt;éclat de volet&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, sur le volet ? Un chat gris se tient sur le pas. Il cligne, les yeux jaunes. Il me regarde, maman. Comme les pommes. Une caisse de pommes attend près du pas de la porte. Les pommes sont jaunes, avec une joue rose. Ça sent le sucré et le bois sec. Elles brillent, maman. Tu les vois, Nino ? Oui, maman. On avance. La cloche de cuivre penche au-dessus du bois. Papa pousse un peu le bois. En ce moment, Nino pousse un peu la porte. La cloche de cuivre fait ding. L'air dedans est frais, un peu sucré. Des bocaux brillent sur une étagère. Je la veux, maintenant. Celle à joue rose ? Oui, tout de suite ! La dame essuie le bois du comptoir. Le chiffon glisse, sans un bruit. Nino se dresse sur les pointes. Une pomme ! Les mots de Nino se cognent au bois. La dame ne lève pas les yeux. Ses mains sont pleines de chiffon. Oh. L'éclat de volet tremble, puis tient. Le sourire de Nino disparaît. Dans sa poitrine, ça se bouscule. L'envie et l'inquiétude se heurtent. Elle ne me voit pas, papa. Ses épaules tombent un peu. Papa se baisse à sa hauteur. La pomme est derrière le bois ? Oui, papa. Nino montre la pomme jaune, à joue rose. Tu parles à la dame, Nino. Le chiffon se pose enfin. La dame lève les yeux. Elle est là. Elle te regarde, Nino ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>bonjour</t>
+          <t>éclat de volet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,39 +1326,66 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_pomme_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un chat gris se tient sur le pas.
-narrateur|Il cligne, tout lent.
-narrateur|Une caisse de pommes sent le sucré.
-narrateur|Les pommes sont jaunes, avec un point rose.
-narrateur|Un volet tape tout doux dans le vent.
-papa|Le chat te regarde, Victorino.
-enfant-m|Il a des yeux jaunes.
+          <t>narrateur|Une poussière claire tombe du volet vert.
+narrateur|Le bois sent le soleil, un peu chaud.
+narrateur|Sur le bois, un éclat de volet luit.
+enfant-m|Il brille, papa.
+papa|Tu le vois, sur le volet ?
+narrateur|Un chat gris se tient sur le pas.
+narrateur|Il cligne, les yeux jaunes.
+enfant-m|Il me regarde, maman.
 maman|Comme les pommes.
-narrateur|Une cloche de cuivre attend au-dessus de la porte.
-narrateur|En ce moment, Victorino pousse un peu.
-narrateur|La cloche fait ding.
+narrateur|Une caisse de pommes attend près du pas de la porte.
+narrateur|Les pommes sont jaunes, avec une joue rose.
+narrateur|Ça sent le sucré et le bois sec.
+enfant-m|Elles brillent, maman.
+maman|Tu les vois, Nino ?
+enfant-m|Oui, maman.
+papa|On avance.
+narrateur|La cloche de cuivre penche au-dessus du bois.
+narrateur|Papa pousse un peu le bois.
+narrateur|En ce moment, Nino pousse un peu la porte.
+narrateur|La cloche de cuivre fait ding.
 narrateur|L'air dedans est frais, un peu sucré.
 narrateur|Des bocaux brillent sur une étagère.
-enfant-m|Une pomme, maman.
-enfant-m|Celle à joue rose.
-maman|On s'approche du comptoir.
+enfant-m|Je la veux, maintenant.
+papa|Celle à joue rose ?
+enfant-m|Oui, tout de suite !
 narrateur|La dame essuie le bois du comptoir.
-narrateur|Le chiffon sent le citron.
-papa|Elle a le chiffon à la main.
-narrateur|Victorino s'arrête devant les pommes.
-narrateur|Le point rose brille sous la lampe.
-narrateur|Un rayon touche le verre des bocaux.
-narrateur|La dame pose le chiffon.
-narrateur|Elle lève les yeux.
-maman|Tu demandes, Victorino.</t>
+narrateur|Le chiffon glisse, sans un bruit.
+narrateur|Nino se dresse sur les pointes.
+enfant-m|Une pomme !
+narrateur|Les mots de Nino se cognent au bois.
+narrateur|La dame ne lève pas les yeux.
+narrateur|Ses mains sont pleines de chiffon.
+enfant-m|Oh.
+narrateur|L'éclat de volet tremble, puis tient.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et l'inquiétude se heurtent.
+enfant-m|Elle ne me voit pas, papa.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|La pomme est derrière le bois ?
+enfant-m|Oui, papa.
+narrateur|Nino montre la pomme jaune, à joue rose.
+maman|Tu parles à la dame, Nino.
+narrateur|Le chiffon se pose enfin.
+narrateur|La dame lève les yeux.
+enfant-m|Elle est là.
+papa|Elle te regarde, Nino ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>cloche,volet</t>
+          <t>volet,cloche</t>
         </is>
       </c>
     </row>
@@ -1385,17 +1412,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Victorino veut la pomme. Que dit-il ?</t>
+          <t>Nino parle à la dame. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorino veut la pomme. Que dit-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino parle à la &lt;emphasis level="moderate"&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand parle à la dame. Quels mots dit-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino parle à la &lt;emphasis&gt;dame&lt;/emphasis&gt;. Quels mots dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1420,7 +1447,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Il dit bonjour. Que dit Victorino ?</t>
+          <t>Il dit bonjour. Quels mots dit-il ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1458,18 +1485,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1484,34 +1511,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>dame</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1520,29 +1551,29 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_parle_a_la_dame_avec_bonjour; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Victorino veut la pomme.
-narrateur|Que dit-il ?</t>
+          <t>narrateur|Nino parle à la dame.
+narrateur|Quels mots dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1569,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une pomme, s'il te plaît. Celle à joue rose. La dame tend une pomme jaune. La peau est lisse, un peu froide. Merci. Merci. Elle a une joue rose. Oui. Tu la tiens des deux mains. Le chat est encore sur le pas. Il ne les suit pas plus loin. Plus tard, l'air change dans la rue. Chez la fleuriste, ça sent fort. Comme un jardin serré. Des tulipes rouges tiennent dans un seau. L'eau tremble un peu. Pour la table. Bonjour. Une fleur, s'il te plaît. La dame tend une tulipe rouge. La tige est lisse, un peu froide. Une goutte glisse le long de la tige. Merci. On la met dans l'eau, à la maison. Victorino porte la pomme. Il porte la tulipe, tout droit.</t>
+          <t>Une pomme. Nino referme la bouche. Nino refuse de foncer. Personne ne parle. Il observe le chiffon, un instant. Il écoute le silence du bois. Bonjour. Bonjour. Une pomme, s'il te plaît. Celle à joue rose. La dame tend une pomme jaune. La peau est lisse, un peu froide. Merci. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle a une joue rose. Tu l'as dans les mains. Nino tourne la pomme, sans se presser. Elle est froide, papa. Oui. On la porte jusqu'à la rue ? Oui, maman. Ils restent un moment près des bocaux. Un rayon touche le verre, étroit. Nino serre la pomme contre lui. On sort ? Oui, papa. Avec la pomme. La cloche de cuivre fait ding.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Bonjour. Bonjour. Une pomme, s'il te plaît. Celle à joue rose. La dame tend une pomme jaune. La peau est lisse, un peu froide. Merci. Merci. Elle a une joue rose. Oui. Tu la tiens des deux mains. Le chat est encore sur le pas. Il ne les suit pas plus loin. Plus tard, l'air change dans la rue. Chez la fleuriste, ça sent fort. Comme un jardin serré. Des tulipes rouges tiennent dans un seau. L'eau tremble un peu. Pour la table. Bonjour. Une fleur, s'il te plaît. La dame tend une tulipe rouge. La tige est lisse, un peu froide. Une goutte glisse le long de la tige. Merci. On la met dans l'eau, à la maison. Victorino porte la pomme. Il porte la tulipe, tout droit.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une pomme. Nino referme la bouche. Nino refuse de foncer. Personne ne parle. Il observe le chiffon, un instant. Il écoute le silence du bois. Bonjour. Bonjour. Une pomme, s'il te plaît. Celle à joue rose. La dame tend une pomme jaune. La peau est lisse, un peu froide. Merci. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle a une joue rose. Tu l'as dans les mains. Nino tourne la pomme, sans se presser. Elle est froide, papa. Oui. On la porte jusqu'à la rue ? Oui, maman. Ils restent un moment près des bocaux. Un rayon touche le verre, étroit. Nino serre la pomme contre lui. On sort ? Oui, papa. Avec la pomme. La cloche de cuivre fait ding.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand a dit &lt;emphasis&gt;bonjour&lt;/emphasis&gt;. Puis s'il te plaît. Puis merci. À l'épicerie, puis chez la fleuriste. [pause]</t>
+          <t>Une pomme. Nino referme la bouche. Nino refuse de foncer. Personne ne parle. Il observe le chiffon, un instant. Il écoute le silence du bois. Bonjour. Bonjour. Une pomme, s'il te plaît. Celle à joue rose. La dame tend une pomme jaune. La peau est lisse, un peu froide. Merci. Merci, Nino. Papa a entendu toute la phrase. Le ventre de Nino se desserre. Les épaules se relèvent un peu. Elle a une joue rose. Tu l'as dans les mains. Nino tourne la pomme, sans se presser. Elle est froide, papa. Oui. On la porte jusqu'à la rue ? Oui, maman. Ils restent un moment près des bocaux. Un rayon touche le verre, étroit. Nino serre la pomme contre lui. On sort ? Oui, papa. Avec la pomme. La cloche de cuivre fait ding. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1626,7 +1657,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1634,10 +1665,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1667,23 +1698,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1692,10 +1723,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1708,44 +1739,47 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=bonjour_s_il_te_plait_merci_vecus; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Bonjour.
+          <t>enfant-m|Une pomme.
+narrateur|Nino referme la bouche.
+narrateur|Nino refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe le chiffon, un instant.
+narrateur|Il écoute le silence du bois.
+enfant-m|Bonjour.
 papa|Bonjour.
 enfant-m|Une pomme, s'il te plaît.
 enfant-m|Celle à joue rose.
 narrateur|La dame tend une pomme jaune.
 narrateur|La peau est lisse, un peu froide.
 enfant-m|Merci.
-maman|Merci.
+papa|Merci, Nino.
+narrateur|Papa a entendu toute la phrase.
+narrateur|Le ventre de Nino se desserre.
+narrateur|Les épaules se relèvent un peu.
 enfant-m|Elle a une joue rose.
+maman|Tu l'as dans les mains.
+narrateur|Nino tourne la pomme, sans se presser.
+enfant-m|Elle est froide, papa.
 papa|Oui.
-maman|Tu la tiens des deux mains.
-narrateur|Le chat est encore sur le pas.
-narrateur|Il ne les suit pas plus loin.
-narrateur|Plus tard, l'air change dans la rue.
-narrateur|Chez la fleuriste, ça sent fort.
-narrateur|Comme un jardin serré.
-narrateur|Des tulipes rouges tiennent dans un seau.
-narrateur|L'eau tremble un peu.
-enfant-m|Pour la table.
-enfant-m|Bonjour.
-enfant-m|Une fleur, s'il te plaît.
-narrateur|La dame tend une tulipe rouge.
-narrateur|La tige est lisse, un peu froide.
-narrateur|Une goutte glisse le long de la tige.
-enfant-m|Merci.
-maman|On la met dans l'eau, à la maison.
-narrateur|Victorino porte la pomme.
-narrateur|Il porte la tulipe, tout droit.</t>
+maman|On la porte jusqu'à la rue ?
+enfant-m|Oui, maman.
+narrateur|Ils restent un moment près des bocaux.
+narrateur|Un rayon touche le verre, étroit.
+narrateur|Nino serre la pomme contre lui.
+papa|On sort ?
+enfant-m|Oui, papa.
+maman|Avec la pomme.
+narrateur|La cloche de cuivre fait ding.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>pomme,cloche</t>
         </is>
       </c>
     </row>
@@ -1772,17 +1806,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>À la maison, maman prend un verre. L'eau fait un petit cercle. La tulipe rouge se tient dedans. Tu veux un bout de pomme ? Oui, papa. S'il te plaît. Victorino croque. C'est croquant. C'est un peu sucré. Merci, papa. Merci, Victorino. La tulipe a encore une goutte. Oui. Dans le verre, maintenant. Le volet tape plus doux, dehors. Le chat n'est plus sur le pas. Il clignait. Tout lent. Un rayon touche encore le verre.</t>
+          <t>Ils passent le pas de la porte. Le volet vert tape une fois. Chez la fleuriste, l'air change. Ça sent fort, comme un jardin serré. Des tulipes rouges tiennent dans l'eau. L'eau tremble un peu, dans le seau. Une tulipe rouge ! Celle-là, bien droite ? Oui, maman. Nino tend la main trop vite. La tige glisse sous ses doigts. La tulipe penche, puis se redresse. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le seau, un instant. Il écoute l'eau, près du bois. Sur le volet vert, l'éclat de volet brille. Bonjour. La dame incline la tête. Une tulipe, s'il te plaît. La dame tend une tulipe rouge. La tige est lisse, un peu froide. Une goutte glisse le long de la tige. Merci. On rentre, maintenant. Tu tiens la pomme des deux mains ? Oui, papa. Nino tient la pomme contre lui. Il tient la tulipe de l'autre main. La tulipe sent le jardin, près du nez.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>À la maison, maman prend un verre. L'eau fait un petit cercle. La tulipe rouge se tient dedans. Tu veux un bout de pomme ? Oui, papa. S'il te plaît. Victorino croque. C'est croquant. C'est un peu sucré. Merci, papa. Merci, Victorino. La tulipe a encore une goutte. Oui. Dans le verre, maintenant. Le volet tape plus doux, dehors. Le chat n'est plus sur le pas. Il clignait. Tout lent. Un rayon touche encore le verre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils passent le pas de la porte. Le volet vert tape une fois. Chez la fleuriste, l'air change. Ça sent fort, comme un jardin serré. Des &lt;emphasis level="moderate"&gt;tulipe&lt;/emphasis&gt;s rouges tiennent dans l'eau. L'eau tremble un peu, dans le seau. Une tulipe rouge ! Celle-là, bien droite ? Oui, maman. Nino tend la main trop vite. La tige glisse sous ses doigts. La tulipe penche, puis se redresse. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le seau, un instant. Il écoute l'eau, près du bois. Sur le volet vert, l'éclat de volet brille. Bonjour. La dame incline la tête. Une tulipe, s'il te plaît. La dame tend une tulipe rouge. La tige est lisse, un peu froide. Une goutte glisse le long de la tige. Merci. On rentre, maintenant. Tu tiens la pomme des deux mains ? Oui, papa. Nino tient la pomme contre lui. Il tient la tulipe de l'autre main. La tulipe sent le jardin, près du nez.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand tient la pomme et la tulipe. Maman dit &lt;emphasis&gt;merci&lt;/emphasis&gt;. [pause]</t>
+          <t>Ils passent le pas de la porte. Le volet vert tape une fois. Chez la fleuriste, l'air change. Ça sent fort, comme un jardin serré. Des &lt;emphasis&gt;tulipe&lt;/emphasis&gt;s rouges tiennent dans l'eau. L'eau tremble un peu, dans le seau. Une tulipe rouge ! Celle-là, bien droite ? Oui, maman. Nino tend la main trop vite. La tige glisse sous ses doigts. La tulipe penche, puis se redresse. Oh. Nino s'arrête. Ses mains se ferment, puis s'ouvrent. Nino refuse de foncer. Personne ne parle. Il observe le seau, un instant. Il écoute l'eau, près du bois. Sur le volet vert, l'éclat de volet brille. Bonjour. La dame incline la tête. Une tulipe, s'il te plaît. La dame tend une tulipe rouge. La tige est lisse, un peu froide. Une goutte glisse le long de la tige. Merci. On rentre, maintenant. Tu tiens la pomme des deux mains ? Oui, papa. Nino tient la pomme contre lui. Il tient la tulipe de l'autre main. La tulipe sent le jardin, près du nez. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1829,7 +1863,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1837,10 +1871,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1863,30 +1897,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>merci</t>
+          <t>tulipe</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1895,10 +1929,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1909,33 +1943,51 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_la_tulipe; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|À la maison, maman prend un verre.
-narrateur|L'eau fait un petit cercle.
-narrateur|La tulipe rouge se tient dedans.
-papa|Tu veux un bout de pomme ?
+          <t>narrateur|Ils passent le pas de la porte.
+narrateur|Le volet vert tape une fois.
+narrateur|Chez la fleuriste, l'air change.
+narrateur|Ça sent fort, comme un jardin serré.
+narrateur|Des tulipes rouges tiennent dans l'eau.
+narrateur|L'eau tremble un peu, dans le seau.
+enfant-m|Une tulipe rouge !
+maman|Celle-là, bien droite ?
+enfant-m|Oui, maman.
+narrateur|Nino tend la main trop vite.
+narrateur|La tige glisse sous ses doigts.
+narrateur|La tulipe penche, puis se redresse.
+enfant-m|Oh.
+narrateur|Nino s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Nino refuse de foncer.
+narrateur|Personne ne parle.
+narrateur|Il observe le seau, un instant.
+narrateur|Il écoute l'eau, près du bois.
+narrateur|Sur le volet vert, l'éclat de volet brille.
+enfant-m|Bonjour.
+narrateur|La dame incline la tête.
+enfant-m|Une tulipe, s'il te plaît.
+narrateur|La dame tend une tulipe rouge.
+narrateur|La tige est lisse, un peu froide.
+narrateur|Une goutte glisse le long de la tige.
+enfant-m|Merci.
+maman|On rentre, maintenant.
+papa|Tu tiens la pomme des deux mains ?
 enfant-m|Oui, papa.
-enfant-m|S'il te plaît.
-narrateur|Victorino croque.
-narrateur|C'est croquant.
-narrateur|C'est un peu sucré.
-enfant-m|Merci, papa.
-maman|Merci, Victorino.
-enfant-m|La tulipe a encore une goutte.
-papa|Oui.
-papa|Dans le verre, maintenant.
-narrateur|Le volet tape plus doux, dehors.
-maman|Le chat n'est plus sur le pas.
-enfant-m|Il clignait.
-papa|Tout lent.
-narrateur|Un rayon touche encore le verre.</t>
+narrateur|Nino tient la pomme contre lui.
+narrateur|Il tient la tulipe de l'autre main.
+narrateur|La tulipe sent le jardin, près du nez.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>verre</t>
+          <t>eau,tulipe</t>
         </is>
       </c>
     </row>
@@ -1962,17 +2014,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La tulipe se tient dans le verre. La pomme a une petite marque. Bonne soirée, Victorino. Elle a une joue rose, ta pomme.</t>
+          <t>Ils rentrent le long du volet vert. Le vent se tait, près du mur. À la maison, maman met la tulipe dans un verre. L'eau fait un petit cercle. Tu veux un bout de pomme ? Oui, maman. Nino croque. C'est croquant, un peu sucré. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le bois. On est bien, ici. Nino pose la pomme près du verre. On le voit, maman. Tu le vois sur le bois ? Oui, l'éclat. La tulipe rouge se tient dans le verre. La joue rose de la pomme brille. L'éclat de volet tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La tulipe se tient dans le verre. La pomme a une petite marque. Bonne soirée, Victorino. Elle a une joue rose, ta pomme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils rentrent le long du volet vert. Le vent se tait, près du mur. À la maison, maman met la tulipe dans un verre. L'eau fait un petit cercle. Tu veux un bout de pomme ? Oui, maman. Nino croque. C'est croquant, un peu sucré. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le bois. On est bien, ici. Nino pose la pomme près du verre. On le voit, maman. Tu le vois sur le bois ? Oui, l'éclat. La tulipe rouge se tient dans le verre. La joue rose de la pomme brille. L'&lt;emphasis level="moderate"&gt;éclat de volet&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils rentrent le long du volet vert. Le vent se tait, près du mur. À la maison, maman met la tulipe dans un verre. L'eau fait un petit cercle. Tu veux un bout de pomme ? Oui, maman. Nino croque. C'est croquant, un peu sucré. Comme tout à l'heure, papa ! Tu le vois, toi ? Oui, sur le bois. On est bien, ici. Nino pose la pomme près du verre. On le voit, maman. Tu le vois sur le bois ? Oui, l'éclat. La tulipe rouge se tient dans le verre. La joue rose de la pomme brille. L'&lt;emphasis&gt;éclat de volet&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2019,18 +2071,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2039,12 +2091,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2053,17 +2105,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de volet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2072,11 +2128,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2085,27 +2141,51 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La tulipe se tient dans le verre.
-narrateur|La pomme a une petite marque.
-maman|Bonne soirée, Victorino.
-papa|Elle a une joue rose, ta pomme.</t>
+          <t>narrateur|Ils rentrent le long du volet vert.
+narrateur|Le vent se tait, près du mur.
+narrateur|À la maison, maman met la tulipe dans un verre.
+narrateur|L'eau fait un petit cercle.
+maman|Tu veux un bout de pomme ?
+enfant-m|Oui, maman.
+narrateur|Nino croque.
+narrateur|C'est croquant, un peu sucré.
+enfant-m|Comme tout à l'heure, papa !
+papa|Tu le vois, toi ?
+enfant-m|Oui, sur le bois.
+maman|On est bien, ici.
+narrateur|Nino pose la pomme près du verre.
+enfant-m|On le voit, maman.
+maman|Tu le vois sur le bois ?
+enfant-m|Oui, l'éclat.
+narrateur|La tulipe rouge se tient dans le verre.
+narrateur|La joue rose de la pomme brille.
+narrateur|L'éclat de volet tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>verre</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2298,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>